<commit_message>
Add JDHG market scan report
</commit_message>
<xml_diff>
--- a/data/findings.xlsx
+++ b/data/findings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -422,7 +422,7 @@
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="33" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
@@ -1911,6 +1911,1203 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>High priority</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Haines Medical Australia</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, infection control, new, mater): Why Haines - Haines Medical Australia</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Haines is a priority competitor for JDHG. The wording suggests a product, catalogue, or availability change that should be verified. The signal mentions a watched hospital or private hospital group. Matched JDHG-relevant terms: patient handling, infection control, new, mater. Evidence snippet: You have no items in your shopping cart. Here are six reasons why you should choose Haines® Medical Australia for your infection control and patient handling equipment:. Haines® Medical Australia is an Australian owned and operated company that has proudly supplied Australia’s Hospitals, Healthcare and Aged Care Facilities, Health Associations and the genera</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Account follow-up</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://hainesmedical.com.au/pages/why-haines</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://hainesmedical.com.au/pages/why-haines</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>High priority</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Haines Medical Australia</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (underpad, ppe, curtain, catalogue, safety): [PDF] Medical Curtains &amp; Tourniquets - ACIPC Conference</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Haines is a priority competitor for JDHG. Matched JDHG-relevant terms: underpad, ppe, curtain, catalogue, safety. Evidence snippet: Medical Curtains &amp; Tourniquets Efficiency, Safety and Care hainesmedical.com.au Haines® Medical Australia’s Single Patient Use Tourniquet offers a simple, cost effective alternative to: • Disposable tourniquets, as they can be used for the duration of the patient’s stay, and most patients find them just as comfortable. Multi-resistant organisms (MROs), inclu</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Update sales collateral</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://acipcconference.com.au/wp-content/uploads/2022/11/ACIPC-Curtains-SPUTS-Catalogue-Nov22.pdf</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://acipcconference.com.au/wp-content/uploads/2022/11/ACIPC-Curtains-SPUTS-Catalogue-Nov22.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Arjo Australia</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, pressure injury, stretcher, new, introducing): Arjo strengthens leading position in patient handling by introducing ...</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, pressure injury, stretcher, new, introducing. Evidence snippet: Pressure Injury Prevention ... Arjo strengthens leading position in patient handling by introducing the new Maxi Move 5 patient floor lift.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://www.arjo.com/en-us/about-us/investors/newsroom/press-releases/2025/5033470-Arjo-strengthens-leading-position-in-patient-handling-by</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://www.arjo.com/en-us/about-us/investors/newsroom/press-releases/2025/5033470-Arjo-strengthens-leading-position-in-patient-handling-by</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>High priority</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Haines Medical Australia</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, infection control, new): Buy Haines Medical Products in Australia</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Haines is a priority competitor for JDHG. The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, infection control, new. Evidence snippet: Haines Medical Australia is an Australian managed company, specializing in infection control and safe patient handling, that has proudly supplied</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://live.joyamedicalsupplies.com.au/brands/haines</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://live.joyamedicalsupplies.com.au/brands/haines</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>High priority</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Haines Medical Australia</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, infection control, new): Haines</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Haines is a priority competitor for JDHG. The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, infection control, new. Evidence snippet: Device Technologies is proud to work with Haines Medical Australia to deliver infection control, patient handling and environmentally friendly consumables for</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://www.device.com.au/our-brands/Haines</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://www.device.com.au/our-brands/Haines</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Novis Healthcare</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (pressure care): Novis Healthcare Pty Ltd</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Matched JDHG-relevant terms: pressure care. Evidence snippet: Healthcare Pty Ltd - Lift, patient transfer, stationary. Alternating-pressure bed mattress overlay system. Overhead track patient lifting/transfer system (</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Compliance review</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://www.tga.gov.au/resources/sponsor/novis-healthcare-pty-ltd</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://www.tga.gov.au/resources/sponsor/novis-healthcare-pty-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Novis Healthcare</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, pressure care, new, available, registered): Molift Smart 150 - Novis Healthcare®</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, pressure care, new, available, registered. Evidence snippet: Molift Smart 150 - Novis Healthcare® Novis Healthcare® 527 subscribers 1 likes 83 views 23 Aug 2022 FOR UPDATES: https://www.youtube.com/c/NovisHealthcareAU?sub_confirmation=1 --- PRODUCT AVAILABLE AT: http://novis.com.au TIMESTAMPS 00:00 - Introduction 00:05 - Features of the product 00:51 - Where and How to buy the product in Australia ____________________</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=szE3SIdwLt4</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=szE3SIdwLt4</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Novis Healthcare</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (pressure care, ppe, new, available): Visit our Showrooms - Novis</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: pressure care, ppe, new, available. Evidence snippet: # Visit our Showrooms. Posted by Novis Admin on **18 Nov 2025**. You are welcome to visit our showrooms, equipped with a large range of assisted daily living aids, mobility and pressure care equipment. Book an appointment with our experienced staff by calling 1300 738 885 for a full demonstration on equipment. – 20/12 Mars Road, Lane Cove West. – 3/59 Easter</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Update sales collateral</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://novis.com.au/resources/news/lane-cove-showroom-now-open</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://novis.com.au/resources/news/lane-cove-showroom-now-open</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Haines Medical Australia</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, new): Haines Medical</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Haines is a priority competitor for JDHG. The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, new. Evidence snippet: Haines Medical Australia is an Australian owned company, supporting infection prevention, safe patient handling and environmental sustainability in</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://shop.aidacare.com.au/collections/haines-medical</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://shop.aidacare.com.au/collections/haines-medical</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Haines Medical Australia</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (underpad, ppe, curtain): Haines Disposable Curtain | Antimicrobial MediCurtains® for sale from Haines Medical Australia - MedicalSearch Australia</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Haines is a priority competitor for JDHG. Matched JDHG-relevant terms: underpad, ppe, curtain. Evidence snippet: All Products &gt; Hospital Equipment &amp; Supplies &gt; Hospital Disposable Curtain. # Haines - Disposable Curtain | Antimicrobial MediCurtains®. ## 3 widths (2.5m to 7.5m), standard 2m drop (or custom cut), 2 hook types (roller or S style), 8 standard colours (including neutrals, blue, lilac and teal) and 3 patterns. Haines® Antimicrobial MediCurtains® are designed </t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://www.medicalsearch.com.au/haines-disposable-curtain-antimicrobial-medicurtains/p/172553</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://www.medicalsearch.com.au/haines-disposable-curtain-antimicrobial-medicurtains/p/172553</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Patient Handling</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, hoist, sling, slide sheet, trolley): Slide &amp; Turn Hoist Sheet - Use a hoist to turn a patient</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, hoist, sling, slide sheet, trolley, new. Evidence snippet: Slide &amp; Turn Hoist Sheet - Use a hoist to turn a patient. # Slide &amp; Turn Hoist Sheet. The Slide &amp; Turn Hoist Sheet is a great way of getting a hoist to do the turning, rather than the carer. This product is an alternative to the Slide &amp; Turn Sheet. * Use a trolley hoist or ceiling hoist to do the turning. * **Slide &amp; Turn Hoist Sheet:** Standard design with </t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://www.pelicanmanufacturing.com.au/product/slide-turn-hoist-sheet</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://www.pelicanmanufacturing.com.au/product/slide-turn-hoist-sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Patient Handling</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, hoist, lifter, sling, slide sheet): Patient Hoists &amp; Slings | Patient Lifting Equipment for Disabled &amp; Elderly - Page 1</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, hoist, lifter, sling, slide sheet, new. Evidence snippet: By utilising patient lifts, slings, and ceiling hoists, the need for strenuous manual lifting and handling is minimised. A patient hoist or sling is a free-standing piece of equipment created to support an individual being transported from one place to another. What types of hoists and slings does Patient Handling offer? We offer a range of products includin</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://www.patienthandling.com.au/c/hoists-slings</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://www.patienthandling.com.au/c/hoists-slings</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Etac</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (positioning, sling, stretcher, new, catalogue): Molift</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The wording suggests a product, catalogue, or availability change that should be verified. The signal mentions a watched hospital or private hospital group. Matched JDHG-relevant terms: positioning, sling, stretcher, new, catalogue, mater. Evidence snippet: YEAR User name / Namn MONTH Barcode according to EAN number Molift RgoSling XXXXXXXX EAN NUMBER (01)0XXXXXXXXXXXXX DK: HMI XXXXX TUMBLEDRY MAX 50ºC /122ºF 60-80ºC 140-176ºF NORMAL DO NOT IRON DO NOT DRYCLEAN DO NOT BLEACH Item no: XXXXXXX Material: Polyester, polyethylene Etac AS, Etac Supply Gjøvik Hadelandsveien 2 N-2816 Gjøvik, Norway Size X (21)XXXXXXXX </t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Account follow-up</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://www.imr.net.au/wp-content/uploads/2022/05/Molift-Catalogue.pdf</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://www.imr.net.au/wp-content/uploads/2022/05/Molift-Catalogue.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>HoverTech</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (positioning, lateral transfer, air-assisted, air assisted, infection control): HoverTech International - HoverMatt Air Transfer System</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Matched JDHG-relevant terms: positioning, lateral transfer, air-assisted, air assisted, infection control, safety. Evidence snippet: HoverMatt, the number one choice of hospitals for lateral patient transfers, further addresses infection control and reprocessing concerns with the **HoverMatt Single Patient Use** Air Transfer System. This inflatable transfer mattress works just like the reusable HoverMatt air transfer system; the mattress - and the patient - float on a cushion of air. By v</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>http://hovertech.com.au/hovermatt-spu.html</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>http://hovertech.com.au/hovermatt-spu.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Arjo Australia</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, positioning, lateral transfer, hoist, sling): In bed and lateral transfer slings for medical hoists - Arjo</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Matched JDHG-relevant terms: patient handling, positioning, lateral transfer, hoist, sling, stretcher. Evidence snippet: Slings for lateral transfer, repositioning in bed, prone positioning and limb lifting. Used in combination with a ceiling or passive floor lift.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://www.arjo.com/en-au/products/patient-handling/slings/in-bed-and-lateral-transfer-slings</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://www.arjo.com/en-au/products/patient-handling/slings/in-bed-and-lateral-transfer-slings</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Aidacare</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, hoist, sling, hospital bed, contract): Manual Handling - Easy &amp; Safe Transfers | Aidacare</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Matched JDHG-relevant terms: patient handling, hoist, sling, hospital bed, contract. Evidence snippet: # Manual Handling. * Manual lifting and moving of patients can be unsafe and lead to injuries. * Special equipment should be used for strain-free handling and transfers. * Aidacare offers a wide range of patient handling equipment. * Equipment designed to ensure easy and safe transfers for both caregivers and patients. * Selection includes lifts, hoists, sli</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Add to tender intelligence</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://www.aidacare.co.nz/products-nz/manual-handling-transfer</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://www.aidacare.co.nz/products-nz/manual-handling-transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Patient Handling</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, hoist, sling, slide sheet, new): Slide Sheets - Novis</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, hoist, sling, slide sheet, new. Evidence snippet: Slide Sheets are an essential solution for healthcare professionals and caregivers seeking a safe and efficient way to move patients. Immedia MultiGlide Nylon Handling Gloves. next icon Product Details Immedia MultiGlide Nylon Slide Sheet with Handles. ## Immedia MultiGlide Nylon Slide Sheet with Handles. next icon Product Details Immedia MultiGlide SG Nylon</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://novis.com.au/category/products/patient-handling-2/slide-sheets</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>https://novis.com.au/category/products/patient-handling-2/slide-sheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Patient Handling</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, hoist, sling, slide sheet, new): Slings - Patient Lifting Hoists</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: patient handling, hoist, sling, slide sheet, new. Evidence snippet: We sell a wide range of superior lift slings in a range of sizes, fabrics and models to suit every patient's needs, younger or elderly.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.aidacare.com.au/products/manual-handling-transfer/slings-patient-lifting-hoists</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>https://www.aidacare.com.au/products/manual-handling-transfer/slings-patient-lifting-hoists</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>HoverTech</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (patient handling, positioning, air-assisted, air assisted, safety): HoverTech International - Australia</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Matched JDHG-relevant terms: patient handling, positioning, air-assisted, air assisted, safety. Evidence snippet: HoverMatt Air Transfer System - Reusable &amp; Single Patient Use | HoverMatt MINI. HoverJack Air Patient Lift | HoverJack Evacuation II. ##### **Australian Site**. HoverTech International is the world leader in air-assisted safe patient handling. HoverTech’s complete portfolio of patient handling, repositioning, and handling products reduces caregiver injury, w</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>http://hovertech.com.au</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>http://hovertech.com.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>HoverTech</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (positioning, lateral transfer, air assisted, sling, mater): Lateral Transfers - HoverTech International</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>The signal mentions a watched hospital or private hospital group. Matched JDHG-relevant terms: positioning, lateral transfer, air assisted, sling, mater. Evidence snippet: # Lateral Transfers. Lateral patient transfers are performed in every hospital unit. Using advanced air technology, the HoverMatt® and HoverSling® products can laterally transfer patients up to 1200 lbs with as little as two caregivers. Patients will have a safe, comfortable and dignified experience on all of HoverTech’s lateral transfer and positioning devi</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Account follow-up</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://hovertechinternational.com/solutions/lateral-transfers</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>https://hovertechinternational.com/solutions/lateral-transfers</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Medium priority</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>HoverTech</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>patient handling and positioning devices; theatre consumables; hospital consumables; underpads</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Possible relevant market signal surfaced (positioning, air-assisted, new): Reduce work-related injuries for caregivers</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>The wording suggests a product, catalogue, or availability change that should be verified. Matched JDHG-relevant terms: positioning, air-assisted, new. Evidence snippet: The HoverMatt air-assisted transfer system includes a range of multifunctional products that make patient transfers, boosting and repositioning easier — at the</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Review product overlap</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Low-Medium: Rule-based triage because Claude did not run. Claude API failed for models: claude-3-5-haiku-latest, claude-3-5-haiku-20241022, claude-3-haiku-20240307</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Competitor website / web search</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://www.etac.com/en-gb/uk/about-us/news-and-social-media/newsroom/2024/hovertech---reduces-work-related-injuries</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>https://www.etac.com/en-gb/uk/about-us/news-and-social-media/newsroom/2024/hovertech---reduces-work-related-injuries</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>